<commit_message>
Require at least 3 photos in both the webform and the XLSForm
Webform (wasa-map.html):
- <input type=file> now accepts multiple files
- New live counter under the input ("N selected, need K more" → "✓")
- Submit validates count >= 3; status line is clear about what's missing
- Result JSON has a photos[] array with per-file metadata
- "Download photos" triggers N spaced downloads named recordid_1.ext,
  recordid_2.ext, ... so they pair with the JSON's photos[].index field

XLSForm (wasa-intervention-form.xlsx, local-only):
- Replaced single image row with photo_1 / photo_2 / photo_3 (all
  required) + photo_4 / photo_5 (optional) under a note header
- Labels guide enumerators on shot variety: overview, detail, context,
  plus extras for beneficiaries / before-after / signage
- Bumped form_id to v2 and version to 2026.05.28.2

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wasa-intervention-form.xlsx
+++ b/wasa-intervention-form.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z.kiala\Documents\water_cycle\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z.kiala\Documents\water_cycle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{542D5B16-47D7-47D7-AE55-FE2BB63FB0C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF8C21E5-5664-435E-91DE-69B7FB04696C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{5D5F3748-DAFD-4827-A51E-48132B110982}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{656C6799-462E-4A6D-BCC2-557CC4DD342B}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="87">
   <si>
     <t>type</t>
   </si>
@@ -148,21 +148,69 @@
     <t>Capture the GPS coordinates of this site</t>
   </si>
   <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>photos_note</t>
+  </si>
+  <si>
+    <t>## Photos (at least 3, must be geotagged)</t>
+  </si>
+  <si>
+    <t>Device location services MUST be enabled so EXIF GPS is written to each photo.</t>
+  </si>
+  <si>
     <t>image</t>
   </si>
   <si>
-    <t>photo</t>
-  </si>
-  <si>
-    <t>Photo of intervention (geotagged)</t>
-  </si>
-  <si>
-    <t>Take the photo with the device camera. Device location services MUST be enabled so EXIF GPS is written to the file.</t>
+    <t>photo_1</t>
+  </si>
+  <si>
+    <t>Photo 1 - Overview</t>
+  </si>
+  <si>
+    <t>Wide shot showing the whole site.</t>
   </si>
   <si>
     <t>max-pixels=2048</t>
   </si>
   <si>
+    <t>photo_2</t>
+  </si>
+  <si>
+    <t>Photo 2 - Detail</t>
+  </si>
+  <si>
+    <t>Close-up of the intervention itself.</t>
+  </si>
+  <si>
+    <t>photo_3</t>
+  </si>
+  <si>
+    <t>Photo 3 - Context</t>
+  </si>
+  <si>
+    <t>Showing the intervention in its surrounding landscape.</t>
+  </si>
+  <si>
+    <t>photo_4</t>
+  </si>
+  <si>
+    <t>Photo 4 (optional)</t>
+  </si>
+  <si>
+    <t>Extra photo - beneficiaries, before/after, signage, anything useful.</t>
+  </si>
+  <si>
+    <t>photo_5</t>
+  </si>
+  <si>
+    <t>Photo 5 (optional)</t>
+  </si>
+  <si>
+    <t>Extra photo.</t>
+  </si>
+  <si>
     <t>comment</t>
   </si>
   <si>
@@ -244,10 +292,10 @@
     <t>WASA Intervention Inventory</t>
   </si>
   <si>
-    <t>wasa_intervention_v1</t>
-  </si>
-  <si>
-    <t>2026.05.28</t>
+    <t>wasa_intervention_v2</t>
+  </si>
+  <si>
+    <t>2026.05.28.2</t>
   </si>
   <si>
     <t>en</t>
@@ -613,16 +661,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99385AB4-D32B-44B2-800E-794F45038E30}">
-  <dimension ref="A1:G12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63D1AEA8-E490-4A79-BF69-B3584A8A2767}">
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="105.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="72.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -785,19 +833,13 @@
       <c r="C11" t="s">
         <v>37</v>
       </c>
-      <c r="D11" t="s">
-        <v>17</v>
-      </c>
       <c r="F11" t="s">
         <v>38</v>
       </c>
-      <c r="G11" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
         <v>40</v>
@@ -806,13 +848,107 @@
         <v>41</v>
       </c>
       <c r="D12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" t="s">
+      <c r="G12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
+      <c r="F15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" t="s">
+        <v>55</v>
+      </c>
+      <c r="G16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" t="s">
+        <v>58</v>
+      </c>
+      <c r="E17" t="s">
         <v>28</v>
       </c>
-      <c r="F12" t="s">
-        <v>43</v>
+      <c r="F17" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -821,7 +957,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3F5A960-5C60-4135-BCE4-BE818ED5FD5B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFBD1968-0C81-4C75-9DCC-6B68690BADFF}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -832,7 +968,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -846,10 +982,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -857,10 +993,10 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -868,10 +1004,10 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -879,10 +1015,10 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -890,10 +1026,10 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -901,10 +1037,10 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C7" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -912,10 +1048,10 @@
         <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -923,10 +1059,10 @@
         <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -935,49 +1071,49 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19E4D84E-C216-488F-9C7F-6898FD03A22D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5023EBA-5FD9-4A94-92A1-EE79071BBC46}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="71.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="E2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add "Other" option to the WASA intervention picker
Webform: extra <option value="other"> at the end of the select with
label "Other (describe in the Type field below)".

XLSForm: matching `other` row in the choices sheet. Survey-row hints
on the intervention and type questions updated to point users at the
Type field when they pick Other. Version bumped to 2026.05.28.3.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wasa-intervention-form.xlsx
+++ b/wasa-intervention-form.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z.kiala\Documents\water_cycle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF8C21E5-5664-435E-91DE-69B7FB04696C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F16ED20-C14F-485A-A608-C3705299E172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{656C6799-462E-4A6D-BCC2-557CC4DD342B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{24EAA487-CC81-403E-BAAF-7584F6353F78}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="89">
   <si>
     <t>type</t>
   </si>
@@ -112,13 +112,13 @@
     <t>minimal</t>
   </si>
   <si>
-    <t>Which of the eight WASA interventions does this site demonstrate?</t>
+    <t>Which of the eight WASA interventions does this site demonstrate? Pick 'Other' if it does not match any.</t>
   </si>
   <si>
     <t>Type / sub-category</t>
   </si>
   <si>
-    <t>Free-text sub-type, e.g. live fencing, cover crop, stone bund, farm pond</t>
+    <t>Free-text sub-type. If intervention is 'Other', describe the intervention here.</t>
   </si>
   <si>
     <t>description</t>
@@ -274,6 +274,12 @@
     <t>H - Climate Information Services</t>
   </si>
   <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t>Other (describe in the Type field)</t>
+  </si>
+  <si>
     <t>form_title</t>
   </si>
   <si>
@@ -295,7 +301,7 @@
     <t>wasa_intervention_v2</t>
   </si>
   <si>
-    <t>2026.05.28.2</t>
+    <t>2026.05.28.3</t>
   </si>
   <si>
     <t>en</t>
@@ -661,7 +667,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63D1AEA8-E490-4A79-BF69-B3584A8A2767}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7529D4A-3BB1-4C82-AE2F-91C2ADAB0825}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -670,7 +676,7 @@
     <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="72.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="95.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -957,8 +963,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFBD1968-0C81-4C75-9DCC-6B68690BADFF}">
-  <dimension ref="A1:C9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B4E0FA6-FEF3-4B63-86A4-FC693BACCEBC}">
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
@@ -1065,13 +1071,24 @@
         <v>76</v>
       </c>
     </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" t="s">
+        <v>78</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5023EBA-5FD9-4A94-92A1-EE79071BBC46}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEF59FE5-BE51-4AFB-A16D-E1B3F44150AA}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1084,36 +1101,36 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mirror the form intro into the KoBo XLSForm as an intro note
New `intro_note` row at the top of the survey sheet displays the same
guidance the webform intro shows: a heading, a sentence on what to do,
and a Before-You-Start line about enabling device location services
before taking photos. Markdown-style **bold** and ## heading are
honoured by KoBo Collect and ODK Collect.

Version bumped to 2026.05.28.4.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wasa-intervention-form.xlsx
+++ b/wasa-intervention-form.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z.kiala\Documents\water_cycle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F16ED20-C14F-485A-A608-C3705299E172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E3B467E-AB94-46FE-83B1-DE7314698FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{24EAA487-CC81-403E-BAAF-7584F6353F78}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{98AECFF5-080F-4D6C-9661-4A32B6F2F451}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="91">
   <si>
     <t>type</t>
   </si>
@@ -85,6 +85,19 @@
     <t>device_id</t>
   </si>
   <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>intro_note</t>
+  </si>
+  <si>
+    <t>## Record a WASA intervention site_x000D_
+_x000D_
+Capture a WASA intervention as you visit it. Select the intervention type, write a short description, capture GPS, and take **at least 3 geotagged photos**. Required fields are marked with *._x000D_
+_x000D_
+**Before you start:** make sure device location services are ON so each photo carries an EXIF GPS tag.</t>
+  </si>
+  <si>
     <t>text</t>
   </si>
   <si>
@@ -148,9 +161,6 @@
     <t>Capture the GPS coordinates of this site</t>
   </si>
   <si>
-    <t>note</t>
-  </si>
-  <si>
     <t>photos_note</t>
   </si>
   <si>
@@ -301,7 +311,7 @@
     <t>wasa_intervention_v2</t>
   </si>
   <si>
-    <t>2026.05.28.3</t>
+    <t>2026.05.28.4</t>
   </si>
   <si>
     <t>en</t>
@@ -351,8 +361,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -667,8 +680,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7529D4A-3BB1-4C82-AE2F-91C2ADAB0825}">
-  <dimension ref="A1:G17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0762B124-EEA5-4F3D-9528-5D400BE593EA}">
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -680,26 +693,26 @@
     <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -735,226 +748,237 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="D6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" t="s">
+      <c r="F7" t="s">
         <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
         <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>20</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="C9" t="s">
         <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" t="s">
         <v>28</v>
-      </c>
-      <c r="F9" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" t="s">
         <v>31</v>
       </c>
-      <c r="C10" t="s">
+      <c r="F10" t="s">
         <v>32</v>
-      </c>
-      <c r="D10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" t="s">
-        <v>33</v>
-      </c>
-      <c r="F10" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
         <v>35</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" t="s">
         <v>36</v>
       </c>
-      <c r="C11" t="s">
+      <c r="F11" t="s">
         <v>37</v>
-      </c>
-      <c r="F11" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" t="s">
         <v>39</v>
       </c>
-      <c r="B12" t="s">
+      <c r="F12" t="s">
         <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" t="s">
-        <v>17</v>
-      </c>
-      <c r="F12" t="s">
-        <v>42</v>
-      </c>
-      <c r="G12" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B13" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" t="s">
         <v>44</v>
       </c>
-      <c r="C13" t="s">
+      <c r="G13" t="s">
         <v>45</v>
-      </c>
-      <c r="D13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F13" t="s">
-        <v>46</v>
-      </c>
-      <c r="G13" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" t="s">
         <v>47</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" t="s">
         <v>48</v>
       </c>
-      <c r="D14" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" t="s">
-        <v>49</v>
-      </c>
       <c r="G14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" t="s">
         <v>50</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" t="s">
         <v>51</v>
       </c>
-      <c r="F15" t="s">
-        <v>52</v>
-      </c>
       <c r="G15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" t="s">
         <v>53</v>
       </c>
-      <c r="C16" t="s">
+      <c r="F16" t="s">
         <v>54</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" t="s">
         <v>55</v>
       </c>
-      <c r="G16" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>56</v>
       </c>
-      <c r="C17" t="s">
+      <c r="F17" t="s">
         <v>57</v>
       </c>
-      <c r="D17" t="s">
+      <c r="G17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
         <v>58</v>
       </c>
-      <c r="E17" t="s">
-        <v>28</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="C18" t="s">
         <v>59</v>
+      </c>
+      <c r="D18" t="s">
+        <v>60</v>
+      </c>
+      <c r="E18" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -963,7 +987,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B4E0FA6-FEF3-4B63-86A4-FC693BACCEBC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{722D1BBA-FD46-4A8E-8591-4592597C06D8}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -972,114 +996,114 @@
     <col min="3" max="3" width="36.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1088,7 +1112,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEF59FE5-BE51-4AFB-A16D-E1B3F44150AA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5059094-DD49-403C-8E66-119B09CCCF2D}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1099,38 +1123,38 @@
     <col min="5" max="5" width="71.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>83</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix _x000D_ artifacts in XLSForm cells (use LF only, never CRLF)
When Excel COM writes a cell containing \r\n (CRLF), the OOXML
serialiser preserves the \r as the escape sequence _x000D_ — which
shows as literal text when the file is opened in KoBo Collect, ODK
Collect, or any non-Excel reader. Office Open XML only treats LF as a
line break inside a cell, so the fix is portable: write LF only.

PowerShell here-strings and double-quoted strings always emit CRLF, so
the script now builds line breaks explicitly with [char]10 (LF). The
intro note label is the only cell with embedded newlines; verified
zero _x000D_ matches in xl/sharedStrings.xml after the regen. Version
bumped to 2026.05.28.5.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wasa-intervention-form.xlsx
+++ b/wasa-intervention-form.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z.kiala\Documents\water_cycle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E3B467E-AB94-46FE-83B1-DE7314698FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F96BBA2-3BEE-4D8A-8465-740DB484EF90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{98AECFF5-080F-4D6C-9661-4A32B6F2F451}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0E82CBD0-98DB-45A7-8BFF-FD603CF9C37C}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -91,10 +91,8 @@
     <t>intro_note</t>
   </si>
   <si>
-    <t>## Record a WASA intervention site_x000D_
-_x000D_
-Capture a WASA intervention as you visit it. Select the intervention type, write a short description, capture GPS, and take **at least 3 geotagged photos**. Required fields are marked with *._x000D_
-_x000D_
+    <t>## Record a WASA intervention site
+Capture a WASA intervention as you visit it. Select the intervention type, write a short description, capture GPS, and take **at least 3 geotagged photos**. Required fields are marked with *.
 **Before you start:** make sure device location services are ON so each photo carries an EXIF GPS tag.</t>
   </si>
   <si>
@@ -311,7 +309,7 @@
     <t>wasa_intervention_v2</t>
   </si>
   <si>
-    <t>2026.05.28.4</t>
+    <t>2026.05.28.5</t>
   </si>
   <si>
     <t>en</t>
@@ -680,7 +678,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0762B124-EEA5-4F3D-9528-5D400BE593EA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6840E34-3AC2-4119-B785-3C48BDD58FB9}">
   <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -987,7 +985,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{722D1BBA-FD46-4A8E-8591-4592597C06D8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE8922A8-A0B9-4C55-9E89-617ABE298078}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1112,7 +1110,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5059094-DD49-403C-8E66-119B09CCCF2D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF4AA86-EE8C-4C0B-9E3D-F26E1BFD3493}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
Add example hint to the Type / sub-category field in both forms
Webform: new <small> under the input listing concrete examples
(Replants tree cover, Minimum tillage, Mulching, Contour bunds, Mulch
strips, Grass tufts, Tied ridges, Soil ripping, Farm pond, Check dam,
Cover crop, Live fencing). The placeholder is also rephrased to lead
with the same examples.

XLSForm: hint column on the `type` row carries the same list so
enumerators see it under the field label in KoBo Collect / ODK Collect.
The "If intervention is 'Other'" instruction is preserved as the tail
of the hint. Version bumped to 2026.05.28.6.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wasa-intervention-form.xlsx
+++ b/wasa-intervention-form.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z.kiala\Documents\water_cycle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F96BBA2-3BEE-4D8A-8465-740DB484EF90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AF5415C-8C6D-4835-ADC4-13C600546398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0E82CBD0-98DB-45A7-8BFF-FD603CF9C37C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{E5D8A89E-677F-4FD0-B97C-11604E60329B}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -129,7 +129,7 @@
     <t>Type / sub-category</t>
   </si>
   <si>
-    <t>Free-text sub-type. If intervention is 'Other', describe the intervention here.</t>
+    <t>Examples: Replants tree cover, Minimum tillage, Mulching, Contour bunds, Mulch strips, Grass tufts, Tied ridges, Soil ripping, Farm pond, Check dam, Cover crop, Live fencing. If intervention is 'Other', describe the intervention here.</t>
   </si>
   <si>
     <t>description</t>
@@ -309,7 +309,7 @@
     <t>wasa_intervention_v2</t>
   </si>
   <si>
-    <t>2026.05.28.5</t>
+    <t>2026.05.28.6</t>
   </si>
   <si>
     <t>en</t>
@@ -678,7 +678,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6840E34-3AC2-4119-B785-3C48BDD58FB9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{474155D3-969C-411B-BB4D-3D65C4139C40}">
   <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -687,7 +687,7 @@
     <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="95.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="210.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -985,7 +985,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE8922A8-A0B9-4C55-9E89-617ABE298078}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E50C1FEB-0B2F-47D3-B7CD-7F6FFC31FFCD}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1110,7 +1110,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF4AA86-EE8C-4C0B-9E3D-F26E1BFD3493}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0720FEC6-9990-4700-BC70-388C8BA43CA1}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>